<commit_message>
Build RFP-008 cover sheet from CORE's real template
The .xlsx copy of the Bluebeam cover-sheet template resolves the one thing
that was reconstructed rather than sourced: openpyxl cannot write legacy .xls,
so the previous cover sheet rebuilt the layout from scratch.

build_att_a_cover.py now loads the template and fills only the cells it
highlights in yellow -- D3, D4, D13, D15, D16, C19, F19 -- refusing any write
outside that set, the same rule build_attachment_a.py follows for the Word
template. Merges, column widths, row heights, the =SUM(F19,F21,F23,F25) total
and the 'list' tab come through unchanged.

Verified: exactly six cells differ from the template, all six highlighted.
Contract amount $1,741,321 still reconciles to the GMP R2 leveling sheet.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L5a7Xc4bv5YukLYTW3W1yn
</commit_message>
<xml_diff>
--- a/02-drafts/RFP-008/New-Com TAB - Att A Review Cover Sheet.xlsx
+++ b/02-drafts/RFP-008/New-Com TAB - Att A Review Cover Sheet.xlsx
@@ -2,62 +2,173 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-60" yWindow="-60" windowWidth="15480" windowHeight="11640" tabRatio="901" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cover sheet" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="contract amount summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="list" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <definedNames>
+    <definedName name="list">list!$B$3:$B$6</definedName>
+    <definedName name="PEs">list!$B$3:$B$6</definedName>
+    <definedName name="PMs">list!$D$3:$D$6</definedName>
+    <definedName name="ProjectEngineers">list!$B$3:$B$6</definedName>
+    <definedName name="review_team">list!#REF!</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'cover sheet'!$A$1:$F$27</definedName>
+  </definedNames>
+  <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0.00;-#,##0.00"/>
+  <numFmts count="5">
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
+    <numFmt numFmtId="168" formatCode="#,##0.00;-#,##0.00"/>
   </numFmts>
-  <fonts count="5">
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
+  <fonts count="16">
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <b val="1"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <family val="2"/>
       <b val="1"/>
       <sz val="14"/>
     </font>
     <font>
+      <name val="Segoe UI"/>
+      <family val="2"/>
       <b val="1"/>
-    </font>
-    <font>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00FF0000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF333333"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FFFF0000"/>
+      <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="22"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -70,25 +181,127 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="14" fontId="13" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="15" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -163,9 +376,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -203,7 +416,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -237,6 +450,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -271,9 +485,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -451,188 +666,319 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F27"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="B2:P27"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9.16796875" defaultRowHeight="14.25"/>
   <cols>
-    <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="0.94140625" customWidth="1" style="21" min="1" max="1"/>
+    <col width="17.2578125" customWidth="1" style="21" min="2" max="2"/>
+    <col width="19.8203125" bestFit="1" customWidth="1" style="21" min="3" max="3"/>
+    <col width="1.6171875" customWidth="1" style="21" min="4" max="4"/>
+    <col width="22.7890625" customWidth="1" style="21" min="5" max="5"/>
+    <col width="21.44140625" customWidth="1" style="21" min="6" max="6"/>
+    <col width="20.765625" bestFit="1" customWidth="1" style="21" min="7" max="7"/>
+    <col width="5.390625" customWidth="1" style="21" min="8" max="8"/>
+    <col width="14.83203125" customWidth="1" style="21" min="9" max="9"/>
+    <col width="13.484375" customWidth="1" style="5" min="10" max="10"/>
+    <col width="5.390625" customWidth="1" style="21" min="11" max="11"/>
+    <col width="9.16796875" customWidth="1" style="21" min="12" max="16384"/>
   </cols>
   <sheetData>
-    <row r="2">
-      <c r="D2" s="1" t="inlineStr">
+    <row r="2" ht="29.25" customHeight="1">
+      <c r="D2" s="36" t="inlineStr">
         <is>
           <t>Attachment A Review Log</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="D3" s="2" t="inlineStr">
+      <c r="G2" s="4" t="n"/>
+    </row>
+    <row r="3" ht="14.25" customHeight="1">
+      <c r="D3" s="37" t="inlineStr">
         <is>
           <t>NCSD - Tonopah High School Sports Field Replacement</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="D4" s="2" t="inlineStr">
+      <c r="G3" s="4" t="n"/>
+    </row>
+    <row r="4" ht="14.1" customHeight="1">
+      <c r="D4" s="37" t="inlineStr">
         <is>
           <t>26-01-019</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="B6" s="3" t="inlineStr">
+      <c r="G4" s="4" t="n"/>
+    </row>
+    <row r="5" ht="21" customHeight="1">
+      <c r="B5" s="15" t="n"/>
+      <c r="L5" s="21" t="n"/>
+      <c r="M5" s="8" t="n"/>
+      <c r="N5" s="8" t="n"/>
+      <c r="O5" s="21" t="n"/>
+      <c r="P5" s="21" t="n"/>
+    </row>
+    <row r="6" ht="18.75" customHeight="1">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>Approved By</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>Approval Stamp</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>Reviewed By</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>Reviewed Stamp</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="4" t="inlineStr">
+      <c r="K6" s="10" t="n"/>
+      <c r="L6" s="21" t="n"/>
+      <c r="M6" s="11" t="n"/>
+      <c r="N6" s="11" t="n"/>
+      <c r="O6" s="11" t="n"/>
+      <c r="P6" s="21" t="n"/>
+    </row>
+    <row r="7" ht="40.5" customHeight="1">
+      <c r="B7" s="31" t="inlineStr">
         <is>
           <t>Project Director</t>
         </is>
       </c>
-      <c r="C7" s="4" t="n"/>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="C7" s="32" t="n"/>
+      <c r="E7" s="13" t="inlineStr">
         <is>
           <t>Project Manager</t>
         </is>
       </c>
-      <c r="F7" s="4" t="n"/>
-    </row>
-    <row r="8">
-      <c r="B8" s="4" t="inlineStr">
+      <c r="F7" s="14" t="n"/>
+      <c r="L7" s="21" t="n"/>
+      <c r="M7" s="15" t="n"/>
+      <c r="N7" s="15" t="n"/>
+      <c r="O7" s="19" t="n"/>
+      <c r="P7" s="21" t="n"/>
+    </row>
+    <row r="8" ht="49.5" customHeight="1">
+      <c r="B8" s="31" t="inlineStr">
         <is>
           <t>General Superintendent</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n"/>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="C8" s="32" t="n"/>
+      <c r="E8" s="17" t="inlineStr">
         <is>
           <t>Superintendent</t>
         </is>
       </c>
-      <c r="F8" s="4" t="n"/>
-    </row>
-    <row r="9">
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Tim Roley or Matt Wade (if over $5M)</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="n"/>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="F8" s="14" t="n"/>
+      <c r="L8" s="21" t="n"/>
+      <c r="M8" s="15" t="n"/>
+      <c r="N8" s="15" t="n"/>
+      <c r="O8" s="19" t="n"/>
+      <c r="P8" s="21" t="n"/>
+    </row>
+    <row r="9" ht="46.5" customHeight="1">
+      <c r="B9" s="31" t="inlineStr">
+        <is>
+          <t>Tim Roley or       Matt Wade                    (if over $5M)</t>
+        </is>
+      </c>
+      <c r="C9" s="32" t="n"/>
+      <c r="E9" s="18" t="inlineStr">
         <is>
           <t>Assistant PM (if applicable)</t>
         </is>
       </c>
-      <c r="F9" s="4" t="n"/>
-    </row>
-    <row r="11">
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Final Session; add Invitees: Anne Tall, Erin Hicks, Kathleen Hamilton, Liz Pippett, Inger Pippett</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="2" t="inlineStr">
+      <c r="F9" s="32" t="n"/>
+      <c r="J9" s="21" t="n"/>
+      <c r="L9" s="21" t="n"/>
+      <c r="M9" s="15" t="n"/>
+      <c r="N9" s="15" t="n"/>
+      <c r="O9" s="19" t="n"/>
+      <c r="P9" s="21" t="n"/>
+    </row>
+    <row r="10" ht="18.75" customHeight="1">
+      <c r="B10" s="15" t="n"/>
+      <c r="C10" s="15" t="n"/>
+      <c r="D10" s="19" t="n"/>
+      <c r="E10" s="15" t="n"/>
+      <c r="F10" s="15" t="n"/>
+      <c r="G10" s="19" t="n"/>
+      <c r="J10" s="21" t="n"/>
+      <c r="L10" s="21" t="n"/>
+      <c r="M10" s="21" t="n"/>
+      <c r="N10" s="21" t="n"/>
+      <c r="O10" s="21" t="n"/>
+      <c r="P10" s="21" t="n"/>
+    </row>
+    <row r="11" ht="18.75" customHeight="1">
+      <c r="B11" s="33" t="inlineStr">
+        <is>
+          <t>Final Session; add Invitees: Anne Tall, Erin Hicks, Kathleen Hamilton, Liz Pippett,  Inger Pippett</t>
+        </is>
+      </c>
+      <c r="G11" s="19" t="n"/>
+      <c r="I11" s="19" t="n"/>
+      <c r="J11" s="21" t="n"/>
+    </row>
+    <row r="12" ht="18.75" customHeight="1">
+      <c r="B12" s="30" t="n"/>
+      <c r="C12" s="30" t="n"/>
+      <c r="D12" s="30" t="n"/>
+      <c r="E12" s="30" t="n"/>
+      <c r="F12" s="30" t="n"/>
+    </row>
+    <row r="13" ht="17.25" customHeight="1">
+      <c r="B13" s="39" t="inlineStr">
         <is>
           <t>Subcontractor:</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="40" t="inlineStr">
         <is>
           <t>New-Com, Inc. (TAB Contractors and MMC, Inc.)</t>
         </is>
       </c>
+      <c r="E13" s="41" t="n"/>
+      <c r="F13" s="41" t="n"/>
+      <c r="H13" s="5" t="n"/>
+    </row>
+    <row r="14" ht="20.25" customHeight="1">
+      <c r="B14" s="20" t="n"/>
+      <c r="C14" s="21" t="n"/>
+      <c r="D14" s="21" t="n"/>
+      <c r="E14" s="21" t="n"/>
+      <c r="F14" s="21" t="n"/>
+      <c r="H14" s="5" t="n"/>
     </row>
     <row r="15">
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="34" t="inlineStr">
         <is>
           <t>Anticipated Material Procurement Date:</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="42" t="inlineStr">
         <is>
           <t>CONFIRM</t>
         </is>
       </c>
-    </row>
-    <row r="16">
-      <c r="B16" t="inlineStr">
+      <c r="E15" s="41" t="n"/>
+      <c r="F15" s="41" t="n"/>
+      <c r="H15" s="5" t="n"/>
+    </row>
+    <row r="16" ht="17.25" customHeight="1">
+      <c r="B16" s="39" t="inlineStr">
         <is>
           <t>Anticipated Start Date:</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D16" s="42" t="inlineStr">
         <is>
           <t>CONFIRM</t>
         </is>
       </c>
+      <c r="E16" s="41" t="n"/>
+      <c r="F16" s="41" t="n"/>
+      <c r="H16" s="5" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="22" t="n"/>
+      <c r="H17" s="43" t="n"/>
+    </row>
+    <row r="18">
+      <c r="H18" s="5" t="n"/>
     </row>
     <row r="19">
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="21" t="inlineStr">
         <is>
           <t>*Phase Code</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="24" t="inlineStr">
         <is>
           <t>02-1000-10000</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" s="25" t="inlineStr">
         <is>
           <t>Dollar Amount</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>$1,741,321.00</t>
-        </is>
-      </c>
+      <c r="F19" s="44" t="n">
+        <v>1741321</v>
+      </c>
+      <c r="H19" s="5" t="n"/>
     </row>
     <row r="20">
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">    *Only one Phase Code Per Subcontractor/Vendor per Tim Roley</t>
         </is>
       </c>
+      <c r="E20" s="25" t="n"/>
+      <c r="H20" s="5" t="n"/>
+    </row>
+    <row r="21">
+      <c r="C21" s="25" t="n"/>
+      <c r="E21" s="25" t="n"/>
+      <c r="F21" s="45" t="n"/>
+      <c r="H21" s="46" t="n"/>
+    </row>
+    <row r="22">
+      <c r="E22" s="25" t="n"/>
+      <c r="H22" s="5" t="n"/>
+    </row>
+    <row r="23">
+      <c r="C23" s="25" t="n"/>
+      <c r="E23" s="25" t="n"/>
+      <c r="F23" s="45" t="n"/>
+      <c r="H23" s="46" t="n"/>
+    </row>
+    <row r="24">
+      <c r="E24" s="25" t="n"/>
+      <c r="H24" s="5" t="n"/>
+    </row>
+    <row r="25">
+      <c r="C25" s="25" t="n"/>
+      <c r="E25" s="25" t="n"/>
+      <c r="F25" s="45" t="n"/>
+      <c r="H25" s="5" t="n"/>
+    </row>
+    <row r="26">
+      <c r="H26" s="5" t="n"/>
     </row>
     <row r="27">
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B27" s="21" t="inlineStr">
         <is>
           <t>TOTAL (should equal contract total)</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>$1,741,321.00</t>
-        </is>
+      <c r="E27" s="38">
+        <f>SUM(F19,F21,F23,F25)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <mergeCells count="11">
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="D3:F3"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="D16:F16"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 
@@ -650,110 +996,169 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="47" t="inlineStr">
         <is>
           <t>How we got to the contract amount — RFP-008 — New-Com, Inc. (TAB Contractors and MMC, Inc.)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="48" t="inlineStr">
         <is>
           <t>Reconciled to GMP R2 leveling sheet tab '8' (Site Demo, Earthwork, Paving &amp; Wet Utilities). The leveling total is SUM of the priced column; values marked with an asterisk on that sheet are options and do not count toward it.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="49" t="inlineStr">
         <is>
           <t>Base Bid — TAB proposal 05.12.26, restated 05.22.26</t>
         </is>
       </c>
-      <c r="B4" s="8" t="n">
+      <c r="B4" s="50" t="n">
         <v>1924851</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="49" t="inlineStr">
         <is>
           <t>Deduct: delete Type II and geofabric from turf field</t>
         </is>
       </c>
-      <c r="B5" s="8" t="n">
+      <c r="B5" s="50" t="n">
         <v>-150000</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="49" t="inlineStr">
         <is>
           <t>Deduct: delete slot / trench drains at track</t>
         </is>
       </c>
-      <c r="B6" s="8" t="n">
+      <c r="B6" s="50" t="n">
         <v>-125000</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="49" t="inlineStr">
         <is>
           <t>Add: additional 8" perforated field drain, south end of field (210 LF)</t>
         </is>
       </c>
-      <c r="B7" s="8" t="n">
+      <c r="B7" s="50" t="n">
         <v>30000</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="49" t="inlineStr">
         <is>
           <t>Deduct: Accepted VE #10 — leave access road as-is (incl. relocation of 2,100 CY to stockpile)</t>
         </is>
       </c>
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="50" t="n">
         <v>-16750</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="49" t="inlineStr">
         <is>
           <t>Add: D-10 dozer for hard dig, 1 month (saves 2 weeks)</t>
         </is>
       </c>
-      <c r="B9" s="8" t="n">
+      <c r="B9" s="50" t="n">
         <v>70000</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="49" t="inlineStr">
         <is>
           <t>Add: trencher for storm drain</t>
         </is>
       </c>
-      <c r="B10" s="8" t="n">
+      <c r="B10" s="50" t="n">
         <v>18720</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="49" t="inlineStr">
         <is>
           <t>Deduct: Accepted VE #9 — RCP flared end section in lieu of headwall</t>
         </is>
       </c>
-      <c r="B11" s="8" t="n">
+      <c r="B11" s="50" t="n">
         <v>-10500</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="51" t="inlineStr">
         <is>
           <t>CONTRACT TOTAL</t>
         </is>
       </c>
-      <c r="B12" s="10" t="n">
+      <c r="B12" s="52" t="n">
         <v>1741321</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
+  <cols>
+    <col width="4.8515625" customWidth="1" min="1" max="1"/>
+    <col width="18.609375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="12.75" customHeight="1">
+      <c r="B2" s="1" t="n"/>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Roger Baum</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+    </row>
+    <row r="4">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Merv Giles</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Matt Buckhannon</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Jim Jacobs</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait"/>
+</worksheet>
 </file>
</xml_diff>